<commit_message>
feat: orkli lookup stable and media download pipeline working
</commit_message>
<xml_diff>
--- a/data/output/reports/lookup_orkli.xlsx
+++ b/data/output/reports/lookup_orkli.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,21 @@
           <t>estado</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>local_image</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>local_pdf</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>media_status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -479,7 +494,11 @@
           <t>E-23758</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>E-23758-00</t>
@@ -511,6 +530,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -523,7 +549,11 @@
           <t>E-23545-00</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>E-23545-00</t>
@@ -555,6 +585,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -567,7 +604,11 @@
           <t>E-3259</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>E-3259-00</t>
@@ -599,6 +640,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -611,7 +659,11 @@
           <t>V-08749-00</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>V-08749-00</t>
@@ -643,6 +695,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -655,7 +714,11 @@
           <t>E-25353-00</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>E-25353-00</t>
@@ -687,6 +750,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -699,7 +769,11 @@
           <t>E-5135</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>E-5135</t>
@@ -731,6 +805,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -743,7 +824,11 @@
           <t>E-5137</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>E-5137</t>
@@ -775,6 +860,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -787,7 +879,11 @@
           <t>E-5139</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>E-5139</t>
@@ -819,6 +915,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -831,7 +934,11 @@
           <t>E-5141</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>E-5141</t>
@@ -863,6 +970,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -875,7 +989,11 @@
           <t>E-5427</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>E-5427</t>
@@ -907,6 +1025,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -919,7 +1044,11 @@
           <t>E-13727</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
           <t>E-13727</t>
@@ -951,6 +1080,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -963,7 +1099,11 @@
           <t>E-13667</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>E-13667</t>
@@ -995,6 +1135,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1007,7 +1154,11 @@
           <t>E-13670</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
           <t>E-13670</t>
@@ -1039,6 +1190,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1051,7 +1209,11 @@
           <t>E-13643</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>E-13643</t>
@@ -1083,6 +1245,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1095,7 +1264,11 @@
           <t>E-13816</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>E-13816</t>
@@ -1127,6 +1300,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1139,7 +1319,11 @@
           <t>E-15700</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>E-15700</t>
@@ -1171,6 +1355,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1183,7 +1374,11 @@
           <t>E-13768</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>E-13768</t>
@@ -1215,6 +1410,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1227,7 +1429,11 @@
           <t>E-18873</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>E-18873</t>
@@ -1259,6 +1465,13 @@
           <t>encontrado</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1271,7 +1484,11 @@
           <t>V-05369</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>V-05369</t>
@@ -1301,6 +1518,13 @@
       <c r="J20" t="inlineStr">
         <is>
           <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>pendiente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
wip: improve orkli ref matching and document extraction
</commit_message>
<xml_diff>
--- a/data/output/reports/lookup_orkli.xlsx
+++ b/data/output/reports/lookup_orkli.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:M99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -596,12 +596,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ORKLI ACC. VALV. MONOTUB PIPA RECTE 1/2 NEGRA 1816</t>
+          <t>ORKLI ACC. VALV. MONOTUB FEMELLA AMB MANIGUET I JUNTA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>E-3259</t>
+          <t>E-23758</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -611,12 +611,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>E-3259-00</t>
+          <t>E-23758-00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>34,88 € 20</t>
+          <t>75,54 € 20</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -651,12 +651,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ORKLI ACC. VALV. MONOTUB VOLANT BLANC AMB CARGOL</t>
+          <t>ORKLI ACC. VALV. MONOTUB PIPA RECTE 1/2 NEGRA 52390</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>V-08749-00</t>
+          <t>E-23545-00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -666,12 +666,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>V-08749-00</t>
+          <t>E-23545-00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>14,00 € 6</t>
+          <t>34,88 € 20</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -706,12 +706,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ORKLI ACC. VOLANT RODÓ AMB TAPA I CARGOL</t>
+          <t>ORKLI ACC. VALV. MONOTUB PIPA RECTE 1/2 NEGRA 1816</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>E-25353-00</t>
+          <t>E-3259</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -721,12 +721,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>E-25353-00</t>
+          <t>E-3259-00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14,67 € 6</t>
+          <t>34,88 € 20</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -761,12 +761,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ORKLI JOC 2 RACCORDS CU 12</t>
+          <t>ORKLI ACC. VALV. MONOTUB VOLANT BLANC AMB CARGOL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>E-5135</t>
+          <t>V-08749-00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -776,23 +776,23 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>E-5135</t>
+          <t>V-08749-00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ACCE.N.TUBO COBRE.D12 Componentes de radiador ACC - Accesorios de unión</t>
+          <t>14,00 € 6</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+          <t>https://www.orkli.com/documents/26715/33991/Orkli%2Btarifa%2Brepuestos%2B2021%2Biraila/deb3b515-a3c0-4fbb-8015-a812a463dc95</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+          <t>https://www.orkli.com/documents/26715/33991/Orkli%2Btarifa%2Brepuestos%2B2021%2Biraila/deb3b515-a3c0-4fbb-8015-a812a463dc95</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -816,12 +816,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ORKLI JOC 2 RACCORDS CU 14</t>
+          <t>ORKLI ACC. VOLANT RODÓ AMB TAPA I CARGOL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>E-5137</t>
+          <t>E-25353-00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -831,23 +831,23 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>E-5137</t>
+          <t>E-25353-00</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ACCE.N.TUBO COBRE D14 Componentes de radiador ACC - Accesorios de unión</t>
+          <t>14,67 € 6</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+          <t>https://www.orkli.com/documents/26715/33991/Orkli%2Btarifa%2Brepuestos%2B2021%2Biraila/deb3b515-a3c0-4fbb-8015-a812a463dc95</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+          <t>https://www.orkli.com/documents/26715/33991/Orkli%2Btarifa%2Brepuestos%2B2021%2Biraila/deb3b515-a3c0-4fbb-8015-a812a463dc95</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -871,12 +871,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ORKLI JOC 2 RACCORDS CU 15</t>
+          <t>ORKLI JOC 2 RACCORDS CU 12</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>E-5139</t>
+          <t>E-5135</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -886,12 +886,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>E-5139</t>
+          <t>E-5135</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ACCESORIO TUBO COBRE D.15 Componentes de radiador ACC - Accesorios de unión</t>
+          <t>ACCE.N.TUBO COBRE.D12 Componentes de radiador ACC - Accesorios de unión</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -926,12 +926,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ORKLI JOC 2 RACCORDS CU 16</t>
+          <t>ORKLI JOC 2 RACCORDS CU 14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>E-5141</t>
+          <t>E-5137</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -941,12 +941,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>E-5141</t>
+          <t>E-5137</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ACCE.N.TUBO COBRE D16 Componentes de radiador ACC - Accesorios de unión</t>
+          <t>ACCE.N.TUBO COBRE D14 Componentes de radiador ACC - Accesorios de unión</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -981,12 +981,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ORKLI JOC 2 RACCORDS CU 18</t>
+          <t>ORKLI JOC 2 RACCORDS CU 15</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>E-5427</t>
+          <t>E-5139</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -996,12 +996,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>E-5427</t>
+          <t>E-5139</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ACCE.N.TUBO COBRE D18 Componentes de radiador ACC - Accesorios de unión</t>
+          <t>ACCESORIO TUBO COBRE D.15 Componentes de radiador ACC - Accesorios de unión</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -1036,12 +1036,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ORKLI JOC 2 RACCORDS MC 16X2</t>
+          <t>ORKLI JOC 2 RACCORDS CU 16</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>E-13727</t>
+          <t>E-5141</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1051,12 +1051,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>E-13727</t>
+          <t>E-5141</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ACCESORIO MULTICAPA Ø16x2 Componentes de radiador ACC - Accesorios de unión</t>
+          <t>ACCE.N.TUBO COBRE D16 Componentes de radiador ACC - Accesorios de unión</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -1091,12 +1091,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ORKLI JOC 2 RACCORDS MC 18X2</t>
+          <t>ORKLI JOC 2 RACCORDS CU 18</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>E-13667</t>
+          <t>E-5427</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1106,12 +1106,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>E-13667</t>
+          <t>E-5427</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>AC.ALUM.D18x2 Componentes de radiador ACC - Accesorios de unión</t>
+          <t>ACCE.N.TUBO COBRE D18 Componentes de radiador ACC - Accesorios de unión</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1146,12 +1146,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ORKLI JOC 2 RACCORDS MC 20X2</t>
+          <t>ORKLI JOC 2 RACCORDS MC 16X2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>E-13670</t>
+          <t>E-13727</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1161,12 +1161,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>E-13670</t>
+          <t>E-13727</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>AC.ALUM.D20x2 Componentes de radiador ACC - Accesorios de unión</t>
+          <t>ACCESORIO MULTICAPA Ø16x2 Componentes de radiador ACC - Accesorios de unión</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1201,12 +1201,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ORKLI JOC 2 RACCORDS MC 20X2,25</t>
+          <t>ORKLI JOC 2 RACCORDS MC 18X2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>E-13643</t>
+          <t>E-13667</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1216,12 +1216,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>E-13643</t>
+          <t>E-13667</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>AC.ALUM.D20x2,25 Componentes de radiador ACC - Accesorios de unión</t>
+          <t>AC.ALUM.D18x2 Componentes de radiador ACC - Accesorios de unión</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1256,12 +1256,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ORKLI JOC 2 RACCORDS PB 15X1.7</t>
+          <t>ORKLI JOC 2 RACCORDS MC 20X2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>E-13816</t>
+          <t>E-13670</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>E-13816</t>
+          <t>E-13670</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ACC.PB Ø15x1.7 Componentes de radiador ACC - Accesorios de unión</t>
+          <t>AC.ALUM.D20x2 Componentes de radiador ACC - Accesorios de unión</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -1311,12 +1311,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ORKLI JOC 2 RACCORDS PB/PEX 16X1,8</t>
+          <t>ORKLI JOC 2 RACCORDS MC 20X2,25</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>E-15700</t>
+          <t>E-13643</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1326,12 +1326,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>E-15700</t>
+          <t>E-13643</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ACC.PER/PEX/PB Ø16x1.8 Componentes de radiador ACC - Accesorios de unión</t>
+          <t>AC.ALUM.D20x2,25 Componentes de radiador ACC - Accesorios de unión</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -1366,12 +1366,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ORKLI JOC 2 RACCORDS PEX 16X2</t>
+          <t>ORKLI JOC 2 RACCORDS PB 15X1.7</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>E-13768</t>
+          <t>E-13816</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1381,12 +1381,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>E-13768</t>
+          <t>E-13816</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ACC.T.PER D16x2 Componentes de radiador ACC - Accesorios de unión</t>
+          <t>ACC.PB Ø15x1.7 Componentes de radiador ACC - Accesorios de unión</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -1421,12 +1421,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ORKLI JOC 2 RACCORDS PEX 20X1,9</t>
+          <t>ORKLI JOC 2 RACCORDS PB/PEX 16X1,8</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>E-18873</t>
+          <t>E-15700</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1436,12 +1436,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>E-18873</t>
+          <t>E-15700</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ACC.T.PER D20x1.9 Componentes de radiador ACC - Accesorios de unión</t>
+          <t>ACC.PER/PEX/PB Ø16x1.8 Componentes de radiador ACC - Accesorios de unión</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -1476,12 +1476,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ORKLI MOTOR SYNCHRON SAMWOO VALVULA ZONA</t>
+          <t>ORKLI JOC 2 RACCORDS PEX 16X2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>V-05369</t>
+          <t>E-13768</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1491,23 +1491,23 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>V-05369</t>
+          <t>E-13768</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>64,97 €</t>
+          <t>ACC.T.PER D16x2 Componentes de radiador ACC - Accesorios de unión</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.orkli.com/documents/26715/33991/Orkli%2Btarifa%2Brepuestos%2B2021%2Biraila/deb3b515-a3c0-4fbb-8015-a812a463dc95</t>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.orkli.com/documents/26715/33991/Orkli%2Btarifa%2Brepuestos%2B2021%2Biraila/deb3b515-a3c0-4fbb-8015-a812a463dc95</t>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1523,6 +1523,3283 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ORKLI JOC 2 RACCORDS PEX 20X1,9</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>E-18873</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>E-18873</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ACC.T.PER D20x1.9 Componentes de radiador ACC - Accesorios de unión</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ORKLI MOTOR SYNCHRON SAMWOO VALVULA ZONA</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>V-05369</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>V-05369</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>64,97 €</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/33991/Orkli%2Btarifa%2Brepuestos%2B2021%2Biraila/deb3b515-a3c0-4fbb-8015-a812a463dc95</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/33991/Orkli%2Btarifa%2Brepuestos%2B2021%2Biraila/deb3b515-a3c0-4fbb-8015-a812a463dc95</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ORKLI PONT PROVA VALVULA MONOTUB</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>E-19863</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>E-19863-00</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>PUENTE DE INSTALACION EMP. Componentes de radiador ACC - Accesorios de unión</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ORKLI JOC 2 RACCORDS INOX EUROCON 3/4 16X1.8</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>V-04226</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>V-04226</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ACC.EUROCONO T.PER D16x1,8 Suelo Radiante</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ORKLI JOC 2 RACCORDS INOX EUROCON 3/4 20X2</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>V-04229</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ORKLI RACOR TERMOSTATIC PER COLECTORS MODULARS</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>E-25092</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>E-25092</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>5,50 €</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/33991/Orkli%2Btarifa%2Brepuestos%2B2021%2Biraila/deb3b515-a3c0-4fbb-8015-a812a463dc95</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/33991/Orkli%2Btarifa%2Brepuestos%2B2021%2Biraila/deb3b515-a3c0-4fbb-8015-a812a463dc95</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ORKLI CAUDALIMETRO GRUPO HIDRAULICO 74400</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>V-03816</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ORKLI ARMARI METAL·LIC EMPOTRAR  840X510X90/130</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1008090</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ORKLI ARMARI PLASTIC 335X275X88</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>E-18620</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>E-18620</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ARMARIO PLÁSTICO 335x275x88 Suelo Radiante</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ORKLI ARMARI PLASTIC 415X275X88</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>E-18621</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>E-18621</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ARMARIO PLÁSTICO 415x275x88 Suelo Radiante</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ORKLI ARMARI PLASTIC 515X275X88</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>E-18622</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>E-18622</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>ARMARIO PLÁSTICO 515x275x88 Suelo Radiante</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ORKLI CAPÇAL TERMOELECTRIC M30X1,5 NC 230V</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>CT410800</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ORKLI CAPÇAL TERMOELECTRIC M30X1,5 NC 230V MICRO</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>V-05001</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>V-05001</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>CAB.TERMOELECTRICA NC230V.M30x1.5 C/MIC Suelo Radiante</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ORKLI COL·LECTOR INOX MUNTAT 3/4 COMPLET 5 SORTIDES</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>SM1005S</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ORKLI COL·LECTOR-VALVULA M-F 3/4-M24X1,5  2 SORTIDES</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>CM35100</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ORKLI COL·LECTOR-VALVULA M-F 3/4-M24X1,5  3 SORTIDES</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>CM35101</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ORKLI COL·LECTOR-VALVULA M-F 3/4-M24X1,5  4 SORTIDES</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>CM35102</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>ORKLI COL·LECTOR-VALVULA M-F 1"-M24X1,5  3 SORTIDES</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>CM35104</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ORKLI COL·LECTOR-VALVULA M-F 1"-M24X1,5  4 SORTIDES</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>CM35105</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ORKLI RACCORD ADAPTADOR CAPÇAL M28X1</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>V-02214</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>V-02214</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>ADAPTADOR M28x1 CABEZA TERMOELECTRICA Suelo Radiante</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ORKLI RACCORD ADAPTADOR CAPÇAL M30X1,5</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>V-02070</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>V-02070</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>ADAPTADOR M30x1.5 CABEZA</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/76863/ORKLI%2BTARIFA%2B2025/eb336f3b-6f15-48c4-a766-4333dc7d33a7</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ORKLI MODUL COL.LECTOR RETORN 2V 1" CS2200</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>CS2200</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ORKLI MODUL COL.LECTOR RETORN 3V 1" CS3200</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>CS3200</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ORKLI MONTURA COL-LECTOR LLAUTO E-24881</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>E-24881</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>E-24881</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>4,47 €</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/33991/Orkli%2Btarifa%2Brepuestos%2B2021%2Biraila/deb3b515-a3c0-4fbb-8015-a812a463dc95</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/documents/26715/33991/Orkli%2Btarifa%2Brepuestos%2B2021%2Biraila/deb3b515-a3c0-4fbb-8015-a812a463dc95</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ORKLI CRONOTERMOSTAT AMBIENT ON-OF RA300</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>RA300</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ORKLI TERMOSTAT AMBIENT DIGITAL ESTIU-HIV. RA210</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>RA210</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ORKLI TERMOSTAT AMBIENT DIGITAL ON-OFF RA200</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>RA200</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ORKLI TERMOSTAT AMBIENT MECANIC ESTIU-HIV. RA110</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>RA110</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ORKLI TERMOSTAT AMBIENT MECANIC ON-OF RA100</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>RA100</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA ZONA CLASICA MICRO 2 VIES  3/4</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>30223200</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA ZONA CLASICA MICRO 2 VIES 1"</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>30323200</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA ZONA CLASICA MICRO 3 VIES  3/4</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>40223200</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA ZONA CLASICA MICRO 3 VIES 1"</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>40323200</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA ZONA CLASICA S/MICRO 2 VIES  1/2</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>30113200</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA ZONA CLASICA S/MICRO 2 VIES  3/4</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>30213200</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA ZONA CLASICA S/MICRO 2 VIES 1"</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>30313200</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA ZONA CLASICA S/MICRO 3VIES  1/2</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>40113200</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA ZONA CLASICA S/MICRO 3VIES  3/4</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>40213200</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA ZONA CLASICA S/MICRO 3 VIES 1"</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>40313200</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ORKLI TUBERIA PEX-A ROTLLE EVOH 16X1.8</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>SRTBA16-200</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ORKLI ACTUADOR VALVULA ZONA NEW AMB MICRO 240V</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>50024200</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>50024200</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>VDZ - Actuador - Con micro NUEVO MODELOR 240V 10</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://files.orkli.com:11443/Fotos_web/50014200.jpg</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/es/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F029/SF034</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ORKLI ACTUADOR VALVULA ZONA NEW S/MICRO 240V</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>50014200</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>50014200</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>VDZ - Actuador - Sin micro NUEVO MODELOR 240V 10</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://files.orkli.com:11443/Fotos_web/50014200.jpg</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/es/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F029/SF034</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ORKLI COS VALVULA ZONA NEW  2 VIES  1/2</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>39104000</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>39104000</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>VDZ - Parte valvular 2 vías - 1/2" Nuevo Modelo 10</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>https://files.orkli.com:11443/Fotos_web/39104000.jpg</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/es/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F029/SF034</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ORKLI COS VALVULA ZONA NEW  2 VIES  3/4</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>39204000</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>39204000</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>VDZ - Parte valvular 2 vías - 3/4" Nuevo Modelo 10</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>https://files.orkli.com:11443/Fotos_web/39104000.jpg</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/es/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F029/SF034</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ORKLI COS VALVULA ZONA NEW  2 VIES   1"</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>39304000</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>39304000</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>VDZ - Parte valvular 2 vías - 1" Nuevo Modelo 10</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>https://files.orkli.com:11443/Fotos_web/39104000.jpg</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/es/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F029/SF034</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>ORKLI COS VALVULA ZONA NEW  3 VIES  1/2</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>49104000</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>49104000</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>VDZ - Parte valvular 3 vías - 1/2" Nuevo Modelo 10</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>https://files.orkli.com:11443/Fotos_web/49104000.jpg</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/es/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F029/SF034</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ORKLI COS VALVULA ZONA NEW  3 VIES  3/4</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>49204000</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>49204000</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>VDZ - Parte valvular 3 vías - 3/4" Nuevo Modelo 10</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>https://files.orkli.com:11443/Fotos_web/49104000.jpg</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/es/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F029/SF034</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>ORKLI COS VALVULA ZONA NEW  3 VIES   1"</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>49304000</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>49304000</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>VDZ - Parte valvular 3 vías - 1" Nuevo Modelo 10</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>https://files.orkli.com:11443/Fotos_web/49104000.jpg</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/es/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F029/SF034</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>ORKLI GRUP SEGURETAT STANDARD RECTE 7K. 3/4</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>GS1110000</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA CALDERA CONNEXIO CALEFACCIO 3/4</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>91399-00</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA SEGURETAT VS 1/2-3K</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>17003-00</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA SEGURETAT VS 1/2-3K AMB TOMA MAN.</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>17004-00</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA SEGURETAT VS 1/2-7K</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>17011-01</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA SEGURETAT VSM 1/2-3K MANOMETRE</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>17004-01</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>ORKLI CAPÇAL TERMOSTATIC HARMONY LX LIQUID</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>60010</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>ORKLI DETENTOR RADIADOR  3/8X12-20 ESC.</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>87210</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>ORKLI DETENTOR RADIADOR 1/2X12-20 ESC.</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1220</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>ORKLI DETENTOR RADIADOR ROSCAR  3/8 ESC.</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1015</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>ORKLI DETENTOR RADIADOR ROSCAR 1/2 ESC.</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1025</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>ORKLI DETENTOR RADIADOR SOLDAR 15X1/2 ESC.</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1425</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA BITUB TERMT. 1/2X12-20 52490</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>52490</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA BITUB TERMT. 1/2X12-20 52720</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>52720</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA MONOTUB NIQ. 1/2 S/REG.</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1816</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>1816</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>VDR MONOT. No Termost. - M 1/2" S. Reglaje 20 33.42</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F027/SF032</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA MONOTUB NIQ. 1/2-18 D/REG.</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1866</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>1866</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>VDR MONOT. No Termost. - M 1/2" Mét.Tubo 26*1,5 - D.Reglaje 20 38.14</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F027/SF032</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA MONOTUB NIQ. 1/2-18 S/REG.</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1817</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>1817</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>VDR MONOT. No Termost. - M 1/2" Mét.Tubo 26*1,5 - S Reglaje 20 33.42</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F027/SF032</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA MONOTUB TERMT. 1/2X12-20 52390</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>52390</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>52390</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>VDR MONOT. Termost. - M 1/2" Espacios Reducidos 20 37.68</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F027/SF032</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA MONOTUB TERMT. 1/2X12-20 52710</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>52710</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>52710</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>VDR MONOT. Termost. - M 1/2" Estandar 20 37.68</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F027/SF032</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA MONOTUB TERMT. D 1/2X12-20 52310</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>52310</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>52310</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>VDR MONOT. Termost. - M 1/2" Toallero Pared Cabz. Drcha. 20 54.72</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F027/SF032</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA MONOTUB TERMT. E 1/2X12-20 52110</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>52110</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>orkli</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>52110</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>VDR MONOT. Termost. - M 1/2" Toallero Pared Cabz. Izda. 20 54.72</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F027/SF032</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>ref_exact</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>encontrado</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA RADIADOR 3/8X12-20 ESC.</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>81210</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA RADIADOR 1/2X12-20 ESC.</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>82210</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA RADIADOR ROSCAR  3/8 ESC.</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1115</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA RADIADOR ROSCAR 1/2 ESC.</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1125</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA RADIADOR SOLDAR 15X1/2 ESC.</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1325</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA RADIADOR TERMT. ROSCAR  3/8 ESC.</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>67150</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA RADIADOR TERMT. ROSCAR 1/2 ESC.</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>67450</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA RADIADOR TERMT. SOLDAR 15X1/2 ESC.</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>67401</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA RADIADOR TERMT. M24X1,5 - 1/2 ESC.</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>67490</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>ORKLI VALVULA RADIADOR TERMT. M24X1,5 - 1/2 ESC. INVERTIDA</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>67690</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>no_match</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>no_encontrado</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr">
         <is>
           <t>pendiente</t>
         </is>

</xml_diff>

<commit_message>
feat: add Playwright PDF fallback for Orkli product docs
</commit_message>
<xml_diff>
--- a/data/output/reports/lookup_orkli.xlsx
+++ b/data/output/reports/lookup_orkli.xlsx
@@ -3529,7 +3529,11 @@
           <t>https://files.orkli.com:11443/Fotos_web/49104000.jpg</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://www.orkli.com/es/web/confortysalud/hidraulica-calefaccion?p_p_id=orklicatalogo_WAR_orkliportlet&amp;p_p_lifecycle=2&amp;p_p_state=normal&amp;p_p_mode=view&amp;p_p_resource_id=documento&amp;p_p_cacheability=cacheLevelPage&amp;_orklicatalogo_WAR_orkliportlet_codigo=187&amp;_orklicatalogo_WAR_orkliportlet_referencia=49204000&amp;_orklicatalogo_WAR_orkliportlet_idFamilia=F029&amp;_orklicatalogo_WAR_orkliportlet_idGranFamilia=2GF015&amp;_orklicatalogo_WAR_orkliportlet_idSubFamilia=SF034&amp;_orklicatalogo_WAR_orkliportlet_idSolCatalogo=HID</t>
+        </is>
+      </c>
       <c r="H67" t="inlineStr">
         <is>
           <t>https://www.orkli.com/es/web/confortysalud/hidraulica-calefaccion/-/cat/HID/2GF015/F029/SF034</t>

</xml_diff>